<commit_message>
data and preprint updated
following the authors' reply on pubpeer and their correction of the discrepencies in the N listed for Zemestani 2020
</commit_message>
<xml_diff>
--- a/data/raw/data_zhao_forest_plot_1_extracted.xlsx
+++ b/data/raw/data_zhao_forest_plot_1_extracted.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10329"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Ian-Hussey/git/verification_zhao_et_al_2023/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94F243B7-B550-5540-9126-C9A5D7DE6D46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{754D02E0-6EC8-5D4F-8F66-65493612F44C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1320" yWindow="500" windowWidth="24580" windowHeight="18380" activeTab="1" xr2:uid="{6C13305E-F56E-F543-B315-2D77D63C8F92}"/>
   </bookViews>
@@ -202,7 +202,7 @@
     <t>checked, correct. However the original summary stats are concerning: SD = 16 is very large for BDI-II given no selection criteria mentioned.</t>
   </si>
   <si>
-    <t>incorrectly extracted. original summary stats are concerning: SD = 3.4 and maybe even 5.15 are very small for BDI-II given their stated selection criteria.</t>
+    <t>original study reports different sample sizes in figure 1 vs table table 2. Figure 1 is more likely to be correct, and is used here. original summary stats are concerning: SD = 3.4 and maybe even 5.15 are very small for BDI-II given their stated selection criteria.</t>
   </si>
 </sst>
 </file>
@@ -251,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -259,7 +259,8 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1227,7 +1228,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:13" s="3" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" s="3" customFormat="1" ht="85" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1238,16 +1239,16 @@
         <v>3.4</v>
       </c>
       <c r="D6" s="5">
-        <v>23</v>
-      </c>
-      <c r="E6" s="2">
+        <v>26</v>
+      </c>
+      <c r="E6" s="6">
         <v>32.57</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="6">
         <v>5.15</v>
       </c>
       <c r="G6" s="5">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H6" s="1" t="b">
         <v>1</v>

</xml_diff>